<commit_message>
add source sentences to pkm symbol review
Each (mission, symbol) row now includes the original sentence(s) from
the SG report that mention the symbol, joined with ¶ separators where
the symbol is cited in multiple paragraphs (e.g. MONUSCO 2808 (2025)
appears in 6 distinct sentences).

Also clarify all rationale text to refer to
data/references/peacekeeping_mission_mandates.csv by name instead of
just "the curated CSV".
</commit_message>
<xml_diff>
--- a/data/processed/pkm2026/pkm_mandate_symbol_review.xlsx
+++ b/data/processed/pkm2026/pkm_mandate_symbol_review.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PKM mandate symbol review'!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PKM mandate symbol review'!$A$1:$H$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,8 @@
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="90" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -529,6 +530,11 @@
           <t>Rationale</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sentence(s) in SG report</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -561,7 +567,14 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2797 (2025), by which it extended the mandate until 31 October 2026.
+---
+The most recent extension of the mandate was authorized by the Council in its resolution 2797 (2025), by which it extended the mandate until 31 October 2026.</t>
         </is>
       </c>
     </row>
@@ -592,7 +605,14 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of MINURSO was established by the Security Council in its resolution 690 (1991).
+---
+The mandate of the United Nations Mission for the Referendum in Western Sahara (MINURSO) was established by the Security Council in its resolution 690 (1991).</t>
         </is>
       </c>
     </row>
@@ -623,7 +643,12 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2703 (2023) and 2756 (2024).</t>
         </is>
       </c>
     </row>
@@ -654,7 +679,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2703 (2023) and 2756 (2024).</t>
         </is>
       </c>
     </row>
@@ -688,6 +718,11 @@
           <t>OIOS establishment statute, cited for OIOS evaluation authority, not MINURSO mandate.</t>
         </is>
       </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>During the 2024/25 period, the Office of Internal Oversight Services conducted an evaluation of MINURSO (IED-24-020) in accordance with General Assembly resolution 48/218 B.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -720,7 +755,14 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of MINUSCA was established by the Security Council in its resolution 2149 (2014).
+---
+The mandate of the United Nations Multidimensional Integrated Stabilization Mission in the Central African Republic (MINUSCA) was established by the Security Council in its resolution 2149 (2014).</t>
         </is>
       </c>
     </row>
@@ -751,7 +793,20 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2800 (2025), by which it extended the mandate until 15 November 2026.
+---
+The most recent extension of the mandate was authorized by the Council in its resolution 2800 (2025), by which the Council extended the mandate until 15 November 2026.
+---
+In its resolution 2800 (2025), the Security Council reduced the authorized strength of the uniformed component of the Mission by deciding that MINUSCA shall comprise up to 14,046 military personnel, including 580 military observers and military staff officers, and 2,999 police personnel, including 589 individual police officers and 2,410 formed police unit personnel, as well as 108 corrections officers, recalled its intention to keep that number under continuous review, taking into account progress on the security situation and the objective of transition and eventual drawdown of MINUSCA when conditions were met, and further expressed its firm intention to review the number of personnel following the successful completion of the electoral process scheduled in 2025 and 2026.
+---
+The successful conduct of the combined presidential, legislative, regional and municipal elections on 28 December 2025 marked a significant milestone for the Central African Republic and provides an opportunity for MINUSCA to adjust its footprint and posture in line with its mandate under Security Council resolution 2800 (2025).
+---
+In the light of the post-election context, and in preparation for implementation of the MINUSCA mandate during the 2026/27 period, the Mission is initiating a phase of consolidation, reconfiguration and internal strategic review, in line with paragraph 48 of Security Council resolution 2800 (2025).</t>
         </is>
       </c>
     </row>
@@ -782,7 +837,12 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2709 (2023) and 2759 (2024).</t>
         </is>
       </c>
     </row>
@@ -813,7 +873,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2709 (2023) and 2759 (2024).</t>
         </is>
       </c>
     </row>
@@ -847,6 +912,11 @@
           <t>GA nationalization request (NPO post justification), not MINUSCA mandate.</t>
         </is>
       </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>In line with the request from the General Assembly in its resolution 76/274 for further nationalization and taking into account the proposed abolishment of one post of Senior Victims’ Rights Officer (P-5) in the Office of the Special Representative of the Secretary-General, the capacity of national staff and the potential for increased efficiencies, it is proposed that one post of Victims’ Rights Officer (National Professional Officer) be established.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -879,7 +949,14 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of MINUSMA was established by the Security Council in its resolution 2100 (2013).
+---
+The mandate of MINUSMA was established by the Security Council in its resolution 2100 (2013) and extended in subsequent resolutions of the Council.</t>
         </is>
       </c>
     </row>
@@ -910,7 +987,16 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>The Security Council, in paragraph 1 of resolution 2690 (2023), decided to terminate the mandate of MINUSMA as from 30 June 2023.
+---
+The mandate for the performance reporting period was provided by the Council in its resolution 2690 (2023).
+---
+The Security Council, in paragraph 1 of resolution 2690 (2023), decided to terminate the mandate of MINUSMA under resolution 2640 (2022) as from 30 June 2023.</t>
         </is>
       </c>
     </row>
@@ -944,6 +1030,11 @@
           <t>Operative mandate at time of termination — cited alongside 2690 in the termination sentence.</t>
         </is>
       </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>The Security Council, in paragraph 1 of resolution 2690 (2023), decided to terminate the mandate of MINUSMA under resolution 2640 (2022) as from 30 June 2023.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -976,7 +1067,14 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of MONUSCO was established by the Security Council in its resolution 1925 (2010).
+---
+The mandate of the United Nations Organization Stabilization Mission in the Democratic Republic of the Congo (MONUSCO) was established by the Security Council in its resolution 1925 (2010).</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1105,16 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>In the 2026/27 period, the strategic priorities of the Mission include the achievement of the objectives set out in Security Council resolution 2773 (2025).
+---
+In the 2026/27 period, the strategic priorities of MONUSCO are expected to contribute to (a) the protection of civilians in its areas of deployment; (b) the achievement of the objectives set out in Security Council resolution 2773 (2025); and (c) support for the stabilization and strengthening of State institutions in the Democratic Republic of the Congo.
+---
+Subsequently, the Security Council, in its resolution 2808 (2025), introduced a new mandate priority for MONUSCO to support the implementation of Council resolution 2773 (2025), with a focus on support for a permanent ceasefire.</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1145,22 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2808 (2025), by which it extended the mandate until 20 December 2026.
+---
+In addition to its continuing support for regional and international peace efforts, under Council resolution 2808 (2025) the Mission was formally authorized to support the implementation of a permanent ceasefire.
+---
+Under Security Council resolution 2808 (2025), MONUSCO is authorized to support the implementation of a permanent ceasefire, including through participation in the Ceasefire Oversight and Verification Mechanism and the provision of technical and logistical support to the Expanded Joint Verification Mechanism Plus.
+---
+MONUSCO will, to the extent possible, leverage existing infrastructure, assets and support arrangements in North Kivu and Ituri, while retaining an ability to scale, reconfigure or redeploy to support ceasefire monitoring and verification activities in South Kivu, as explicitly authorized in resolution 2808 (2025).
+---
+The Mission will sustain its logistical support for the forward force headquarters in Beni to facilitate joint operations and strengthened coordination with FARDC, while remaining agile and flexible to expand its areas of support to South Kivu, pursuant to Security Council resolution 2808 (2025).
+---
+Subsequently, the Security Council, in its resolution 2808 (2025), introduced a new mandate priority for MONUSCO to support the implementation of Council resolution 2773 (2025), with a focus on support for a permanent ceasefire.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1191,12 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2717 (2023) and 2765 (2024).</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1227,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2717 (2023) and 2765 (2024).</t>
         </is>
       </c>
     </row>
@@ -1135,7 +1267,14 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>The Regional Service Centre in Entebbe (RSCE) was established in July 2010, by the General Assembly in its resolution 64/269, as a shared service centre for missions in the region.
+---
+The Regional Service Centre in Entebbe, Uganda (RSCE), was established in July 2010, by the General Assembly in its resolution 64/269, as a shared service centre for missions in the region under the global field support strategy.</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1305,16 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>The Centre's mandate was expanded to provide additional services to other entities, including the African Union, following the adoption by the General Assembly of its resolution 78/294.
+---
+The Centre’s mandate was expanded to provide additional services to other entities, as well as to develop broader cooperation with regional organizations, such as the African Union, following the adoption by the General Assembly of its resolution 78/294.
+---
+Following the adoption by the General Assembly of its resolution 78/294, RSCE will lead the consolidation of administrative and financial services, excluding payroll, for 16 active clients of the Kuwait Joint Support Office.</t>
         </is>
       </c>
     </row>
@@ -1200,6 +1348,11 @@
           <t>Gave RSCE operational/managerial independence — a substantive mandate change; old ACABQ data included it. Currently not in curated CSV.</t>
         </is>
       </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>In its resolution 69/307, the General Assembly decided to give RSCE operational and managerial independence and requested that the Secretary-General submit a budget proposal for the Centre for the period from 1 July 2016 to 30 June 2017, to be charged against the client missions.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr"/>
@@ -1231,6 +1384,11 @@
           <t>Approved payroll-services consolidation — could be read as a mandate-broadening decision.</t>
         </is>
       </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>32–39), the consolidation of payroll services was approved by the General Assembly in its resolution 80/242.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr"/>
@@ -1262,6 +1420,11 @@
           <t>Terminates UNITAMS (client mission), not RSCE.</t>
         </is>
       </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Effective 1 July 2026, RSCE will assume responsibility for the provision of residual liquidation support to the United Nations Investigative Team to Promote Accountability for Crimes Committed by Da’esh/Islamic State in Iraq and the Levant, whose mandate was terminated by the Security Council in its resolution 2697 (2023), as from 17 September 2024, and the United Nations Assistance Mission for Iraq (UNAMI), whose mandate was terminated by the Council, in its resolution 2732 (2024), as from 31 December 2025.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr"/>
@@ -1293,6 +1456,11 @@
           <t>Terminates UNAMI (client mission), not RSCE.</t>
         </is>
       </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Effective 1 July 2026, RSCE will assume responsibility for the provision of residual liquidation support to the United Nations Investigative Team to Promote Accountability for Crimes Committed by Da’esh/Islamic State in Iraq and the Levant, whose mandate was terminated by the Security Council in its resolution 2697 (2023), as from 17 September 2024, and the United Nations Assistance Mission for Iraq (UNAMI), whose mandate was terminated by the Council, in its resolution 2732 (2024), as from 31 December 2025.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr"/>
@@ -1324,6 +1492,11 @@
           <t>Terminates UNSOM (a client mission), not RSCE's mandate.</t>
         </is>
       </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>The Centre made a smooth transition to supporting the United Nations Transitional Assistance Mission in Somalia after the United Nations Assistance Mission in Somalia ended its operations on 31 October 2024 pursuant to Security Council resolution 2753 (2024).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr"/>
@@ -1355,6 +1528,11 @@
           <t>Nationalization-of-posts policy reference, not RSCE mandate.</t>
         </is>
       </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>In line with General Assembly resolutions 70/286 and 76/274, RSCE has continued to advance the nationalization of posts, supporting the professional growth of the local workforce and strengthening long-term sustainability.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr"/>
@@ -1386,6 +1564,11 @@
           <t>Omnibus GA peacekeeping financing/staffing resolution, not RSCE mandate.</t>
         </is>
       </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>In line with General Assembly resolutions 70/286 and 76/274, RSCE has continued to advance the nationalization of posts, supporting the professional growth of the local workforce and strengthening long-term sustainability.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr"/>
@@ -1417,6 +1600,11 @@
           <t>Endorses ACABQ recommendations on staff movement actions.</t>
         </is>
       </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>15) and endorsed by the General Assembly in its resolution 77/306, are presented in table 2.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr"/>
@@ -1448,6 +1636,11 @@
           <t>Budget transfer of tenant units, not RSCE mandate.</t>
         </is>
       </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>The budgets of tenant units were transferred to their parent offices under the support account, effective from the 2025/26 period, as approved by the General Assembly in its resolution 79/300.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr"/>
@@ -1479,6 +1672,17 @@
           <t>Parser artifact: a sentence/table-cell read as a symbol.</t>
         </is>
       </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>1
+---
+International
+---
+National
+---
+Uniformed</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1511,7 +1715,14 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2811 (2025), by which it extended the Force's mandate until 30 June 2026.
+---
+The most recent extension of the mandate was authorized by the Council in its resolution 2811 (2025), by which it extended the Force’s mandate until 30 June 2026.</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1753,14 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of the United Nations Disengagement Observer Force (UNDOF) was established by the Security Council in its resolution 350 (1974).
+---
+The mandate of the United Nations Disengagement Observation Force (UNDOF) was established by the Security Council in its resolution 350 (1974).</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1791,12 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2737 (2024) and 2766 (2024).</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1827,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2737 (2024) and 2766 (2024).</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1867,12 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of UNFICYP was established by the Security Council in its resolution 186 (1964).</t>
         </is>
       </c>
     </row>
@@ -1670,7 +1903,12 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2815 (2026), by which it extended the mandate until 31 January 2027.</t>
         </is>
       </c>
     </row>
@@ -1704,6 +1942,11 @@
           <t>WPS thematic SC res cited in planning section as framework.</t>
         </is>
       </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Pursuant to Security Council resolution 1325 (2000) and all subsequent resolutions on women and peace and security, UNFICYP will continue to support efforts for the full, meaningful and effective participation of women in peace and political processes and to bring together a broader range of women actors on both sides.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr"/>
@@ -1732,7 +1975,12 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2674 (2023) and 2723 (2024).</t>
         </is>
       </c>
     </row>
@@ -1763,7 +2011,12 @@
       </c>
       <c r="G40" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2674 (2023) and 2723 (2024).</t>
         </is>
       </c>
     </row>
@@ -1797,6 +2050,11 @@
           <t>SC res on civil-society engagement; cited in planning section as operative directive.</t>
         </is>
       </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>The Security Council, in its resolution 2771 (2025), urged the leaders to increase their support to, and ensure a meaningful role for, civil society engagement in peace efforts, in particular strengthening the participation of women’s organizations and young people in the process.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr"/>
@@ -1828,6 +2086,11 @@
           <t>GA staffing-review directive (civilian staffing review), not UNFICYP mandate.</t>
         </is>
       </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>The Force and the Department of Operational Support conducted a civilian staffing review in the 2024/25 period pursuant to General Assembly resolution 76/274.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1860,7 +2123,26 @@
       </c>
       <c r="G43" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>The mandate was expanded by the Security Council in its resolution 1701 (2006).
+---
+The mandate of the United Nations Interim Force in Lebanon (UNIFIL) was established by the Security Council in its resolutions 425 (1978) and 426 (1978), expanded in its resolution 1701 (2006) and extended in subsequent resolutions.
+---
+The subsequent announcement of a cessation of hostilities between Lebanon and Israel (see S/2024/870), effective 27 November 2024, created a period of new opportunities for the implementation of resolution 1701 (2006), with the parties committing to its full implementation.
+---
+Until 27 November 2024, with the movement of UNIFIL highly restricted, the Force’s operational priorities were monitoring violations of resolution 1701 (2006), with significantly increased reporting requirements, as well as liaison and coordination between the parties.
+---
+UNIFIL finalized its adaptation plan in January 2025 and subsequently implemented a more robust, operations-centred modus operandi, with dedicated operations involving multiple military assets, focused on assisting the Lebanese Armed Forces in deploying south of the Litani River, creating a safe and secure environment and preventing violations of resolution 1701 (2006).
+---
+UNIFIL will, during the first six months of the 2026/27 period, prioritize activities aimed at supporting the parties in maintaining the cessation of hostilities and stability along the Blue Line, recommitting to the full implementation of resolution 1701 (2006) and taking concrete steps towards addressing outstanding provisions of that resolution, including steps towards a permanent ceasefire, and a long-term political solution between Lebanon and Israel, which are key to long-term stability.
+---
+UNIFIL will continue to monitor, investigate and report on violations of resolution 1701 (2006), concurrently supporting the parties in fulfilling their commitments to the resolution.
+---
+UNIFIL will intensify its support to the Lebanese Armed Forces to ensure their effective and sustainable deployment south of the Litani River and to enhance their capacities to implement Security Council resolution 1701 (2006).</t>
         </is>
       </c>
     </row>
@@ -1891,7 +2173,22 @@
       </c>
       <c r="G44" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2790 (2025), by which it extended the mandate for a final time until 31 December 2026.
+---
+The most recent extension of the mandate was authorized by the Council in its resolution 2790 (2025), by which it extended the mandate for a final time until 31 December 2026, when the Force is to cease its operations and to start from this date and within one year its orderly and safe drawdown and withdrawal of personnel.
+---
+Pursuant to resolution 2790 (2025), UNIFIL will also remain ready to support, when relevant, enhanced diplomatic efforts to resolve any dispute or reservations pertaining to the international border between Lebanon and Israel.
+---
+UNIFIL will cooperate with and support the mechanism set out in resolution 2790 (2025), including through the Force’s monitoring and verification role.
+---
+A lean and essential leadership and coordination structure of the executive direction and management component will continue to provide unified oversight, ensuring that political, operational and administrative activities remain fully aligned with Security Council resolution 2790 (2025), the directives of the Secretary-General and the relevant policies of the Organization.
+---
+Strategic communications will continue to manage the Force’s public narrative and legacy messaging, countering disinformation and misinformation and ensuring transparent engagement with host authorities and the public, including as provided for under Council resolution 2790 (2025).</t>
         </is>
       </c>
     </row>
@@ -1922,7 +2219,14 @@
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of the United Nations Interim Force in Lebanon (UNIFIL) was established by the Security Council in its resolutions 425 (1978) and 426 (1978).
+---
+The mandate of the United Nations Interim Force in Lebanon (UNIFIL) was established by the Security Council in its resolutions 425 (1978) and 426 (1978), expanded in its resolution 1701 (2006) and extended in subsequent resolutions.</t>
         </is>
       </c>
     </row>
@@ -1953,7 +2257,14 @@
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of the United Nations Interim Force in Lebanon (UNIFIL) was established by the Security Council in its resolutions 425 (1978) and 426 (1978).
+---
+The mandate of the United Nations Interim Force in Lebanon (UNIFIL) was established by the Security Council in its resolutions 425 (1978) and 426 (1978), expanded in its resolution 1701 (2006) and extended in subsequent resolutions.</t>
         </is>
       </c>
     </row>
@@ -1984,7 +2295,12 @@
       </c>
       <c r="G47" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided by the Council in its resolutions 2695 (2023) and 2749 (2024).</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2331,12 @@
       </c>
       <c r="G48" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided by the Council in its resolutions 2695 (2023) and 2749 (2024).</t>
         </is>
       </c>
     </row>
@@ -2049,6 +2370,11 @@
           <t>Parser artifact: a sentence/table-cell read as a symbol.</t>
         </is>
       </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>All parties will remain committed to the implementation of Security Council resolution 1701 (2006); UNIFIL will be afforded freedom of movement by all parties</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2081,7 +2407,14 @@
       </c>
       <c r="G50" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of UNISFA was established by the Security Council in its resolution 1990 (2011).
+---
+The mandate of the United Nations Interim Security Force for Abyei (UNISFA) was established by the Security Council in its resolution 1990 (2011) and extended in subsequent resolutions.</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2445,14 @@
       </c>
       <c r="G51" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2802 (2025), by which it extended the mandate until 15 November 2026.
+---
+In accordance with Security Council resolution 2802 (2025), by which the Council extended the Force’s mandate until 15 November 2026, UNISFA will prepare an additional report for the Council on security situation activities undertaken by authorities in the Sudan and South Sudan to assess demonstrable progress towards achieving benchmarks outlined by the Council, and it will provide a comprehensive assessment of the security implications of any potential drawdown.</t>
         </is>
       </c>
     </row>
@@ -2143,7 +2483,12 @@
       </c>
       <c r="G52" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided by the Council in its resolutions 2708 (2023) and 2760 (2024).</t>
         </is>
       </c>
     </row>
@@ -2174,7 +2519,12 @@
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided by the Council in its resolutions 2708 (2023) and 2760 (2024).</t>
         </is>
       </c>
     </row>
@@ -2208,6 +2558,11 @@
           <t>GA staffing-review directive, not UNISFA mandate.</t>
         </is>
       </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>During the first half of the 2025/26 period, a civilian staffing review was conducted by UNISFA and the Department of Operational Support, in accordance with paragraph 28 of General Assembly resolution 76/274.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2240,7 +2595,12 @@
       </c>
       <c r="G55" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>In its resolution 49/233 A of 23 December 1994, the General Assembly welcomed the establishment of the first permanent United Nations logistics base in Brindisi, Italy, to support peacekeeping operations.</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2631,14 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>In its resolution 63/262 of 24 December 2008, the General Assembly approved the establishment of site B, in Valencia, Spain, as a secondary active telecommunications and information technology facility.
+---
+Subsequently, in its resolution 63/262 of 24 December 2008, the General Assembly approved the establishment of site B, in Valencia, Spain, as a secondary active telecommunications and information technology facility to strengthen operational resilience and ensure business continuity in support of peacekeeping activities.</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2656,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>(only in curated)</t>
+          <t>(only in curated CSV)</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
@@ -2302,7 +2669,12 @@
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV; not picked up by broad extractor.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV); was not picked up by the broad extractor.</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>UNLB is mandated to serve all field missions, Secretariat entities, and United Nations system entities, pursuant to General Assembly resolution 72/266 B on shifting the management paradigm in the United Nations.</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2705,16 @@
       </c>
       <c r="G58" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>The Advisory Committee's recommendations were endorsed by the General Assembly in its resolution 78/295.
+---
+44) endorsed by the Assembly in its resolution 78/295.
+---
+), endorsed by the General Assembly in its resolution 78/295, planning assumptions for strategic deployment stocks had been revised.</t>
         </is>
       </c>
     </row>
@@ -2367,6 +2748,11 @@
           <t>GA directive on UN-AU cooperation; cited in section D (regional cooperation) as programmatic frame.</t>
         </is>
       </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>In 2026/27, the Base will enhance collaboration with regional organizations, in particular the African Union, to improve operational synergies, innovation and joint capabilities in line with General Assembly resolution 79/329.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr"/>
@@ -2398,6 +2784,11 @@
           <t>Same resolution as 72/266 B but normalized without the section letter; collapsed into the curated 72/266 B row.</t>
         </is>
       </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>As part of the Department of Operational Support, UNLB is mandated to serve all field missions, all Secretariat entities, and United Nations system entities, as well as to cooperate in developing broader cooperation with regional organizations, in alignment with the Department’s mandate under the guidance of the Office of Supply Chain Management, pursuant to General Assembly resolution 72/266 B on shifting the management paradigm in the United Nations and the recommendation of the Advisory Committee (A/78/744/Add.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr"/>
@@ -2429,6 +2820,13 @@
           <t>GA budget transfer of tenant units to parent offices; not a UNLB mandate.</t>
         </is>
       </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>The budgets of tenant units and the regional aviation safety office were transferred to their respective parent offices under the support account for peacekeeping operations, effective from the 2025/26 period, as approved by the General Assembly in its resolution 79/300.
+---
+31) endorsed by the General Assembly in its resolution 79/300.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2461,7 +2859,12 @@
       </c>
       <c r="G62" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of UNMIK was established by the Security Council in its resolution 1244 (1999).</t>
         </is>
       </c>
     </row>
@@ -2495,6 +2898,11 @@
           <t>WPS thematic SC res cited in mandate paragraph as cross-cutting framework.</t>
         </is>
       </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>In implementing those priorities, the Mission ensured the integration of gender and youth perspectives into all aspects of its work, in accordance with Security Council resolutions 1325 (2000) and 2250 (2015) and subsequent resolutions on women and peace and security and on youth, peace and security, respectively.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr"/>
@@ -2526,6 +2934,11 @@
           <t>YPS thematic SC res cited in mandate paragraph as cross-cutting framework.</t>
         </is>
       </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>In implementing those priorities, the Mission ensured the integration of gender and youth perspectives into all aspects of its work, in accordance with Security Council resolutions 1325 (2000) and 2250 (2015) and subsequent resolutions on women and peace and security and on youth, peace and security, respectively.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr"/>
@@ -2557,6 +2970,11 @@
           <t>Omnibus GA peacekeeping financing/staffing resolution, not UNMIK mandate.</t>
         </is>
       </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>During the 2025/26 period, a civilian staffing review of UNMIK was undertaken in line with General Assembly resolution 76/274.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2589,7 +3007,14 @@
       </c>
       <c r="G66" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of UNMISS was established by the Security Council in its resolution 1996 (2011).
+---
+The mandate of United Nations Mission in South Sudan (UNMISS) was established by the Security Council in its resolution 1996 (2011).</t>
         </is>
       </c>
     </row>
@@ -2620,7 +3045,14 @@
       </c>
       <c r="G67" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2779 (2025), by which it extended the mandate until 30 April 2026.
+---
+The mandate for the performance period was provided in its resolutions 2729 (2024), 2778 (2025) and 2779 (2025).</t>
         </is>
       </c>
     </row>
@@ -2651,7 +3083,12 @@
       </c>
       <c r="G68" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2729 (2024), 2778 (2025) and 2779 (2025).</t>
         </is>
       </c>
     </row>
@@ -2682,7 +3119,12 @@
       </c>
       <c r="G69" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2729 (2024), 2778 (2025) and 2779 (2025).</t>
         </is>
       </c>
     </row>
@@ -2716,6 +3158,13 @@
           <t>GA staffing-review/nationalization directive, not UNMISS mandate.</t>
         </is>
       </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>During the 2025/26 period, the Mission conducted a civilian staffing review, in accordance with paragraph 28 of General Assembly resolution 76/274.
+---
+In line with the request from the General Assembly in its resolution 76/274 for further nationalization and taking into account both the capacity of national staff and the potential for increased efficiencies, the civilian staffing review recommended six nationalizations through the conversion of posts and positions.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2748,7 +3197,18 @@
       </c>
       <c r="G71" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>The mandate of UNSOH was established by the Security Council in its resolution 2793 (2025).
+---
+The Security Council noted the assessment by the Secretary-General, contained in his letter to the President of the Security Council (S/2025/122), that a United Nations support office should provide comprehensive logistical and operational support to the Gang Suppression Force and, owing to the unique character of the Force, requested the Secretary-General to establish the United Nations Support Office in Haiti (UNSOH) to provide support, primarily to the Gang Suppression Force, the United Nations Integrated Office in Haiti (BINUH), the Haitian National Police and the Haitian Armed Forces on any joint operations with the Gang Suppression Force, as well as technical support to the Organization of American States (OAS), with a view to assuming full logistical support responsibility for the Gang Suppression Force within six months of the adoption of resolution 2793 (2025).
+---
+Through its resolution 2793 (2025), the Security Council established UNSOH as a separate entity in Haiti, with dedicated leadership.
+---
+The requirements take into account the milestones outlined in resolution 2793 (2025), including the provision of support to Gang Suppression Force starting on 1 April 2026 and the anticipated deployment of the Force.</t>
         </is>
       </c>
     </row>
@@ -2779,7 +3239,14 @@
       </c>
       <c r="G72" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>UNSOH will provide mission support services to BINUH in support of the delivery of its mandate, as extended in resolution 2814 (2026).
+---
+UNSOH will provide, on a cost-recovery basis, the standard range of mission support services to BINUH in support of the delivery of its mandate, as extended in resolution 2814 (2026), with a view to assuming full responsibility by 1 February 2026.</t>
         </is>
       </c>
     </row>
@@ -2813,6 +3280,11 @@
           <t>Predecessor MSSM authorization; cited in UNSOH A.Mandate as historical context being transitioned.</t>
         </is>
       </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>In the resolution, the Council authorized Member States to transition the Multinational Security Support Mission, as authorized in resolution 2699 (2023) and renewed in resolution 2751 (2024), to the Gang Suppression Force, in close cooperation and coordination with the Government of Haiti, for an initial period of 12 months, comprising an authorized personnel ceiling of 5,550 for the Gang Suppression Force, consisting of 5,500 uniformed personnel, comprising both military and police personnel, and 50 civilians.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="3" t="inlineStr"/>
@@ -2844,6 +3316,11 @@
           <t>Predecessor MSSM renewal; same context as 2699.</t>
         </is>
       </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>In the resolution, the Council authorized Member States to transition the Multinational Security Support Mission, as authorized in resolution 2699 (2023) and renewed in resolution 2751 (2024), to the Gang Suppression Force, in close cooperation and coordination with the Government of Haiti, for an initial period of 12 months, comprising an authorized personnel ceiling of 5,550 for the Gang Suppression Force, consisting of 5,500 uniformed personnel, comprising both military and police personnel, and 50 civilians.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2876,7 +3353,14 @@
       </c>
       <c r="G75" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>UNSOS was established by the Security Council in its resolution 1863 (2009) to provide support to the African Union Mission in Somalia.
+---
+The United Nations Support Office in Somalia (UNSOS) was established by the Security Council in its resolution 1863 (2009) to provide support to the African Union Mission in Somalia.</t>
         </is>
       </c>
     </row>
@@ -2894,7 +3378,7 @@
       </c>
       <c r="D76" s="3" t="inlineStr">
         <is>
-          <t>(only in curated)</t>
+          <t>(only in curated CSV)</t>
         </is>
       </c>
       <c r="E76" s="3" t="n">
@@ -2907,7 +3391,12 @@
       </c>
       <c r="G76" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV; not picked up by broad extractor.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV); was not picked up by the broad extractor.</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>The United Nations Guard Unit was authorized by the Security Council in its resolution 2124 (2013).</t>
         </is>
       </c>
     </row>
@@ -2938,7 +3427,18 @@
       </c>
       <c r="G77" s="3" t="inlineStr">
         <is>
-          <t>In curated CSV.</t>
+          <t>Kept in data/references/peacekeeping_mission_mandates.csv (the curated CSV).</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>The most recent extension of the mandate was authorized by the Council in its resolution 2809 (2025), by which it extended the mandate until 31 December 2026.
+---
+The Council, in its resolution 2809 (2025), also reaffirmed the continued role of UNSOS in providing required logistical and administrative services, including to the United Nations Transitional Assistance Mission in Somalia (UNTMIS) on a cost-recovery basis until the conclusion of its phased drawdown by 31 October 2026.
+---
+In this context, and consistent with paragraph 23 of resolution 2809 (2025), UNSOS will continue to adapt its support for AUSSOM, taking into account measures implemented to manage its liquidity shortfall and prioritizing the sustained capacity of AUSSOM to consolidate peace and security gains across phases 2, 3 and 4 of the concept of operations.
+---
+Pursuant to resolution 2809 (2025), the implementation of the human rights due diligence policy remains mandatory for all United Nations support provided to AUSSOM and Somali security forces.</t>
         </is>
       </c>
     </row>
@@ -2969,7 +3469,12 @@
       </c>
       <c r="G78" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2748 (2024), 2767 (2024) and 2776 (2025).</t>
         </is>
       </c>
     </row>
@@ -3003,6 +3508,11 @@
           <t>Terminates UNTMIS (the mission UNSOS supports) — drives UNSOS transition role; cited in planning section.</t>
         </is>
       </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>In its resolution 2753 (2024), the Security Council expressed its intention to terminate the mandate of UNTMIS at the end of the anticipated two-phased transition on 31 October 2026.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr"/>
@@ -3031,7 +3541,14 @@
       </c>
       <c r="G80" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2748 (2024), 2767 (2024) and 2776 (2025).
+---
+These positions had been dedicated to providing administrative and operational support to UNTMIS on a cost-recovery basis in accordance with Security Council resolution 2767 (2024).</t>
         </is>
       </c>
     </row>
@@ -3062,12 +3579,17 @@
       </c>
       <c r="G81" s="3" t="inlineStr">
         <is>
-          <t>Performance-period renewal — deliberately dropped from curated per founding+latest rule; defensible to include for completeness.</t>
+          <t>Performance-period renewal — deliberately dropped from the curated CSV per founding+latest rule; defensible to include for completeness.</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>The mandate for the performance period was provided in its resolutions 2748 (2024), 2767 (2024) and 2776 (2025).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:H81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>